<commit_message>
更新 2026-08-21 風險新聞明細（2026-09-03 10:00）
</commit_message>
<xml_diff>
--- a/risk_news_daily/2026-08-21.xlsx
+++ b/risk_news_daily/2026-08-21.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="風險新聞" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'風險新聞'!$A$1:$O$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'風險新聞'!$A$1:$P$83</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O83"/>
+  <dimension ref="A1:P83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -446,6 +446,7 @@
     <col width="80" customWidth="1" min="13" max="13"/>
     <col width="22" customWidth="1" min="14" max="14"/>
     <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -524,6 +525,11 @@
           <t>已人工覆核</t>
         </is>
       </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>曝險金額</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -562,15 +568,13 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>違約</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="n">
-        <v>5</v>
-      </c>
+          <t>一般公司更新</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>通知、檢視授信及自營部位、持續追蹤</t>
+          <t>排除、不納入風險事件</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -589,6 +593,9 @@
         </is>
       </c>
       <c r="O2" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P2" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -629,15 +636,13 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>違約</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="n">
-        <v>5</v>
-      </c>
+          <t>一般公司更新</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>通知、檢視授信及自營部位、持續追蹤</t>
+          <t>排除、不納入風險事件</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -656,6 +661,9 @@
         </is>
       </c>
       <c r="O3" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P3" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -725,6 +733,9 @@
       <c r="O4" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P4" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -792,6 +803,9 @@
       <c r="O5" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P5" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -859,6 +873,9 @@
       <c r="O6" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P6" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -926,6 +943,9 @@
       <c r="O7" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P7" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -949,11 +969,7 @@
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
+      <c r="F8" s="2" t="inlineStr"/>
       <c r="G8" s="2" t="inlineStr">
         <is>
           <t>LEGAL</t>
@@ -993,6 +1009,9 @@
         </is>
       </c>
       <c r="O8" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="P8" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1062,6 +1081,9 @@
       <c r="O9" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P9" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1129,6 +1151,9 @@
       <c r="O10" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P10" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1196,6 +1221,9 @@
       <c r="O11" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P11" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1263,6 +1291,9 @@
       <c r="O12" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P12" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1330,6 +1361,9 @@
       <c r="O13" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P13" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1397,6 +1431,9 @@
       <c r="O14" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P14" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1464,6 +1501,9 @@
       <c r="O15" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P15" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1531,6 +1571,9 @@
       <c r="O16" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P16" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1598,6 +1641,9 @@
       <c r="O17" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P17" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1665,6 +1711,9 @@
       <c r="O18" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P18" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1732,6 +1781,9 @@
       <c r="O19" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P19" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1755,11 +1807,7 @@
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
+      <c r="F20" s="2" t="inlineStr"/>
       <c r="G20" s="2" t="inlineStr">
         <is>
           <t>LEGAL</t>
@@ -1799,6 +1847,9 @@
         </is>
       </c>
       <c r="O20" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="P20" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1868,6 +1919,9 @@
       <c r="O21" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P21" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1935,6 +1989,9 @@
       <c r="O22" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P22" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2002,6 +2059,9 @@
       <c r="O23" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P23" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2069,6 +2129,9 @@
       <c r="O24" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P24" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2136,6 +2199,9 @@
       <c r="O25" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P25" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2159,11 +2225,7 @@
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
+      <c r="F26" s="2" t="inlineStr"/>
       <c r="G26" s="2" t="inlineStr">
         <is>
           <t>LEGAL</t>
@@ -2203,6 +2265,9 @@
         </is>
       </c>
       <c r="O26" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="P26" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2272,6 +2337,9 @@
       <c r="O27" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P27" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2339,6 +2407,9 @@
       <c r="O28" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P28" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2406,6 +2477,9 @@
       <c r="O29" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P29" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2473,6 +2547,9 @@
       <c r="O30" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P30" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2540,6 +2617,9 @@
       <c r="O31" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P31" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2607,6 +2687,9 @@
       <c r="O32" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P32" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2674,6 +2757,9 @@
       <c r="O33" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P33" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2741,6 +2827,9 @@
       <c r="O34" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P34" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2808,6 +2897,9 @@
       <c r="O35" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P35" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2875,6 +2967,9 @@
       <c r="O36" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P36" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2942,6 +3037,9 @@
       <c r="O37" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P37" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3009,6 +3107,9 @@
       <c r="O38" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P38" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3076,6 +3177,9 @@
       <c r="O39" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P39" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3143,6 +3247,9 @@
       <c r="O40" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P40" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3210,6 +3317,9 @@
       <c r="O41" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P41" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3277,6 +3387,9 @@
       <c r="O42" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P42" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3344,6 +3457,9 @@
       <c r="O43" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P43" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3411,6 +3527,9 @@
       <c r="O44" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P44" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3478,6 +3597,9 @@
       <c r="O45" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P45" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3545,6 +3667,9 @@
       <c r="O46" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P46" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3612,6 +3737,9 @@
       <c r="O47" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P47" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3679,6 +3807,9 @@
       <c r="O48" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P48" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3746,6 +3877,9 @@
       <c r="O49" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P49" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3813,6 +3947,9 @@
       <c r="O50" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P50" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3880,6 +4017,9 @@
       <c r="O51" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P51" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3945,6 +4085,9 @@
         </is>
       </c>
       <c r="O52" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P52" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4012,6 +4155,9 @@
         </is>
       </c>
       <c r="O53" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P53" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4081,6 +4227,9 @@
       <c r="O54" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P54" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -4148,6 +4297,9 @@
       <c r="O55" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P55" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -4215,6 +4367,9 @@
       <c r="O56" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P56" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -4282,6 +4437,9 @@
       <c r="O57" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P57" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -4305,11 +4463,7 @@
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr"/>
-      <c r="F58" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
+      <c r="F58" s="2" t="inlineStr"/>
       <c r="G58" s="2" t="inlineStr">
         <is>
           <t>MARKET</t>
@@ -4349,6 +4503,9 @@
         </is>
       </c>
       <c r="O58" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="P58" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4418,6 +4575,9 @@
       <c r="O59" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P59" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -4485,6 +4645,9 @@
       <c r="O60" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P60" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -4552,6 +4715,9 @@
       <c r="O61" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P61" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -4619,6 +4785,9 @@
       <c r="O62" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P62" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -4686,6 +4855,9 @@
       <c r="O63" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P63" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -4753,6 +4925,9 @@
       <c r="O64" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P64" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -4820,6 +4995,9 @@
       <c r="O65" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P65" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -4887,6 +5065,9 @@
       <c r="O66" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P66" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -4954,6 +5135,9 @@
       <c r="O67" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P67" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -5021,6 +5205,9 @@
       <c r="O68" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P68" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -5088,6 +5275,9 @@
       <c r="O69" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P69" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -5155,6 +5345,9 @@
       <c r="O70" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P70" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -5222,6 +5415,9 @@
       <c r="O71" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P71" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -5289,6 +5485,9 @@
       <c r="O72" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P72" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -5356,6 +5555,9 @@
       <c r="O73" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P73" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -5423,6 +5625,9 @@
       <c r="O74" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P74" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -5490,6 +5695,9 @@
       <c r="O75" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P75" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -5555,6 +5763,9 @@
         </is>
       </c>
       <c r="O76" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P76" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5622,6 +5833,9 @@
         </is>
       </c>
       <c r="O77" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P77" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5691,6 +5905,9 @@
       <c r="O78" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P78" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -5758,6 +5975,9 @@
       <c r="O79" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P79" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -5825,6 +6045,9 @@
       <c r="O80" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P80" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -5892,6 +6115,9 @@
       <c r="O81" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P81" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -5959,6 +6185,9 @@
       <c r="O82" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P82" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -6026,9 +6255,12 @@
       <c r="O83" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="P83" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O83"/>
+  <autoFilter ref="A1:P83"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>